<commit_message>
Dashboard 2026-08-27 + файлы лотов
</commit_message>
<xml_diff>
--- a/vse-loti/339193000/spec-339193000.xlsx
+++ b/vse-loti/339193000/spec-339193000.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -497,13 +497,50 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>комплект со склада СОТ (шкаф, ИБП с картой мониторинга, АВР – новые на складе СОТ), смонтировать по проекту с переносом линий. Доукомплектовать шкаф «грозозацитой SNR-SPNet-PRM24-v2» и 3 модулями «Грозозащита Ethernet SNR-SPNet-BP1100», патч панелью ( cabeus 7955 c + 7962 c или аналог) (Приложение 2 ) . Видеокамеру CAM-66-ST подключить с использование POE удлинителя. POE удлинитель разместить в боксе, в доступном месте, на высоте 1,5 м. Предусмотреть доукомплектование узлов связи N узла ИБП (оборудование Заказчика) Грозозащита SNR-SPNet-PRM24-v2» и модули Ethernet SNR-SPNet-BP1100» (оборудование Подрядчика) Патч панель (cabeus 7955c + 7962c или аналог) (оборудование Подрядчика) N01 + N02 + + + N04 + + + N10 + + + Требования к архитектурно-строительным, объемно-планировочным и конструктивным решениям Не требуется Требования к режиму безопасности и гигиене труда Технические решения должны соответствовать требованиям экономических, санитарно-гигиенических, противопожарных и других норм, действующих на территории Российской Федерации, и обеспечивать безопасную для жизни и здоровья людей эксплуатацию объекта. Устанавливаемое на объекте оборудование должно быть безвредно для здоровья лиц, имеющих доступ на объект. Требования и условия для разработки природоохранных мер и мероприятий Не требуется . Требования по разработке инженерно-технических мероприятий по гражданской обороне и предупреждению чрезвычайных ситуаций Не требуется . Требования по выполнению исследований и конструкторских разработок Не требуется . Требования к проведению, оформлению и представлению расчета стоимости строительства Локально сметный расчет выполнить ресурсно-индексным методом в федеральной сметно-нормативной базе ФСНБ 2022 г. Для материалов отсутствующих в сметно-нормативной базе, в расчете предоставить конъюнктурный анализ с предоставлением не менее трех прайсов на каждую позицию материалов поставщиков Челябинской области. Особые условия Не требуются . Перечень технических регламентов и стандартов, норм и правил, соответствие которым необходимо обеспечить при проектировании ГОСТ Р 21.1101-20 20 СПДС. Основные требования к проектной и рабочей документации (с Поправкой) ГОСТ Р 21.101-2020 СПДС. Спецификация оборудования, изделий и материалов. ГОСТ Р 53246-2008 Информационные технологии (ИТ). Системы кабельные структурированные. Проектирование основных узлов системы. Общие требования. ГОСТ Р 53245-2008. Информационные технологии. Системы кабельные структурированные. Монтаж основных узлов системы. Методы испытания. Правила по охране труда при эксплуатации электроустановок Правила по охране труда при выполнении работ на объектах связи Перечень согласований и экспертиз в государственных федеральных и региональных надзорных органах Не требуется . Требования к процедуре подтверждения соответствия проекта Заданию на проектирование Внутренняя экспертиза Заказчика (ПСД и проектных решений) . Требования к телекоммуникационной инфраструктуре Для подключения проектируемого объекта к сети передачи данных запросить технические условия в управлении ИТ филиала ПАО «ТМК» ЧТПЗ на этапе проектирования. Проектирование и строительство объекта выполнить в соответствии с типовыми требованиями ИТ к телекоммуникационной инфраструктуре. (приложение 3 ), если иное не указано в данном задании. Требование к оборудованию охранного телевидения Требования к камерам Модель/количество видеокамер: Внутренняя IP-видеокамера Dahua DH-IPC-HDW3449HP-AS-PV-0280B-PRO</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>шт</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="H2" s="2" t="n">
+      <c r="H3" s="2" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Источник: 851900595.txt</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>